<commit_message>
fix issue with ps plots
</commit_message>
<xml_diff>
--- a/app/data/smd.xlsx
+++ b/app/data/smd.xlsx
@@ -402,7 +402,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>arrhythmia_base</t>
+          <t>arrhythmia</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -422,7 +422,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>pacemaker_base</t>
+          <t>pacemaker</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -442,7 +442,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>hyperlipidemia_base</t>
+          <t>hyperlipidemia</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -462,7 +462,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>hypertension_base</t>
+          <t>hypertension</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -482,7 +482,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>depression_base</t>
+          <t>depression</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -502,7 +502,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>epilepsy_base</t>
+          <t>epilepsy</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>cardio_base</t>
+          <t>cardio</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>cvd_base</t>
+          <t>cvd</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -562,7 +562,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ihd_base</t>
+          <t>ihd</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>pvd_base</t>
+          <t>pvd</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>vhd_base</t>
+          <t>vhd</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>hepatic_base</t>
+          <t>hepatic</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>acute_renal_base</t>
+          <t>acute_renal</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chronic_renal_base</t>
+          <t>chronic_renal</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>hypokalemia_base</t>
+          <t>hypokalemia</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>hypocalcemia_base</t>
+          <t>hypocalcemia</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>hypomagnesemia_base</t>
+          <t>hypomagnesemia</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>stroke_base</t>
+          <t>stroke</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>copd_base</t>
+          <t>copd</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>mi_base</t>
+          <t>mi</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>suicidal_base</t>
+          <t>suicidal</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>chf_base</t>
+          <t>chf</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>arrhythmia_base</t>
+          <t>arrhythmia</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>pacemaker_base</t>
+          <t>pacemaker</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>hyperlipidemia_base</t>
+          <t>hyperlipidemia</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>hypertension_base</t>
+          <t>hypertension</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>depression_base</t>
+          <t>depression</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>epilepsy_base</t>
+          <t>epilepsy</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>cardio_base</t>
+          <t>cardio</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>cvd_base</t>
+          <t>cvd</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ihd_base</t>
+          <t>ihd</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>pvd_base</t>
+          <t>pvd</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>vhd_base</t>
+          <t>vhd</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>hepatic_base</t>
+          <t>hepatic</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>acute_renal_base</t>
+          <t>acute_renal</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>chronic_renal_base</t>
+          <t>chronic_renal</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>hypokalemia_base</t>
+          <t>hypokalemia</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>hypocalcemia_base</t>
+          <t>hypocalcemia</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>hypomagnesemia_base</t>
+          <t>hypomagnesemia</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>stroke_base</t>
+          <t>stroke</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>copd_base</t>
+          <t>copd</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>mi_base</t>
+          <t>mi</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>suicidal_base</t>
+          <t>suicidal</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>chf_base</t>
+          <t>chf</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>arrhythmia_base</t>
+          <t>arrhythmia</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>pacemaker_base</t>
+          <t>pacemaker</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>hyperlipidemia_base</t>
+          <t>hyperlipidemia</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>hypertension_base</t>
+          <t>hypertension</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>depression_base</t>
+          <t>depression</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>epilepsy_base</t>
+          <t>epilepsy</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>cardio_base</t>
+          <t>cardio</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>cvd_base</t>
+          <t>cvd</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ihd_base</t>
+          <t>ihd</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>pvd_base</t>
+          <t>pvd</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>vhd_base</t>
+          <t>vhd</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>hepatic_base</t>
+          <t>hepatic</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>acute_renal_base</t>
+          <t>acute_renal</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>chronic_renal_base</t>
+          <t>chronic_renal</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>hypokalemia_base</t>
+          <t>hypokalemia</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>hypocalcemia_base</t>
+          <t>hypocalcemia</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>hypomagnesemia_base</t>
+          <t>hypomagnesemia</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>stroke_base</t>
+          <t>stroke</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>copd_base</t>
+          <t>copd</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>mi_base</t>
+          <t>mi</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>suicidal_base</t>
+          <t>suicidal</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>chf_base</t>
+          <t>chf</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>arrhythmia_base</t>
+          <t>arrhythmia</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>pacemaker_base</t>
+          <t>pacemaker</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>hyperlipidemia_base</t>
+          <t>hyperlipidemia</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>hypertension_base</t>
+          <t>hypertension</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>depression_base</t>
+          <t>depression</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>epilepsy_base</t>
+          <t>epilepsy</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>cardio_base</t>
+          <t>cardio</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>cvd_base</t>
+          <t>cvd</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ihd_base</t>
+          <t>ihd</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>pvd_base</t>
+          <t>pvd</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>vhd_base</t>
+          <t>vhd</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>hepatic_base</t>
+          <t>hepatic</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>acute_renal_base</t>
+          <t>acute_renal</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>chronic_renal_base</t>
+          <t>chronic_renal</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>hypokalemia_base</t>
+          <t>hypokalemia</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2322,7 +2322,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>hypocalcemia_base</t>
+          <t>hypocalcemia</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>hypomagnesemia_base</t>
+          <t>hypomagnesemia</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>stroke_base</t>
+          <t>stroke</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>copd_base</t>
+          <t>copd</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>mi_base</t>
+          <t>mi</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>suicidal_base</t>
+          <t>suicidal</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>chf_base</t>
+          <t>chf</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>arrhythmia_base</t>
+          <t>arrhythmia</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>pacemaker_base</t>
+          <t>pacemaker</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>hyperlipidemia_base</t>
+          <t>hyperlipidemia</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>hypertension_base</t>
+          <t>hypertension</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>depression_base</t>
+          <t>depression</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>epilepsy_base</t>
+          <t>epilepsy</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>cardio_base</t>
+          <t>cardio</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>cvd_base</t>
+          <t>cvd</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>ihd_base</t>
+          <t>ihd</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>pvd_base</t>
+          <t>pvd</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>vhd_base</t>
+          <t>vhd</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>hepatic_base</t>
+          <t>hepatic</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>acute_renal_base</t>
+          <t>acute_renal</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>chronic_renal_base</t>
+          <t>chronic_renal</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>hypokalemia_base</t>
+          <t>hypokalemia</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>hypocalcemia_base</t>
+          <t>hypocalcemia</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>hypomagnesemia_base</t>
+          <t>hypomagnesemia</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>stroke_base</t>
+          <t>stroke</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>copd_base</t>
+          <t>copd</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>mi_base</t>
+          <t>mi</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>suicidal_base</t>
+          <t>suicidal</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>chf_base</t>
+          <t>chf</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">

</xml_diff>